<commit_message>
conversion DOCX => WATM and manifest generation work
</commit_message>
<xml_diff>
--- a/ner/specs/persons-merged.xlsx
+++ b/ner/specs/persons-merged.xlsx
@@ -2190,7 +2190,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Arcivescovo elettore di Magonza; arcivescovo di Magonza; elettor di Magonza; elettore di Magonza</t>
+          <t>Arcivescovo elettore di Magonza; arcivescovato di Magonza; arcivescovo di Magonza; elettor di Magonza; elettore di Magonza</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2759,7 +2759,7 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ambasciator Trivesano; ambasciator Trivisano; ambasciator Trivisiano; eccellentissimo Trevisano; eccellentissimo Trivisano</t>
+          <t>ambasciator Trevisan; ambasciator Trivesano; ambasciator Trivisan; ambasciator Trivisan l; ambasciator Trivisano; ambasciator Trivisiano; eccellentissimo Trevisano; eccellentissimo Trivisano</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3039,7 +3039,7 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Quast; capitan Quast; capitano Quast</t>
+          <t>Quast; capitan Quast; capitano Quast; capitano Quest</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -5736,7 +5736,7 @@
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Pieter Milander; Pietro Melander; Pietro Milander; colonello Milander; monsignor Milaender; monsignor Milander; monsignor Miler; signor Milander; signor colonello de ’ Svizzeri Milander</t>
+          <t>Pieter Milander; Pietro Melander; Pietro Milander; collonello Milander; colonello Milan; colonello Milander; monsignor Milaender; monsignor Milander; monsignor Miler; signor Milander; signor colonello de ’ Svizzeri Milander</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -10244,7 +10244,7 @@
       <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Lambert Charles; colonello Lambert Charles</t>
+          <t>Lambert Carles; Lambert Charles; colonello Lambert Charles</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -14568,7 +14568,7 @@
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr">
         <is>
-          <t>duca di Virtembergh; duca di Wirtembergh; duca di Wirtimbergh</t>
+          <t>duca di Virtembergh; duca di Vitembergh; duca di Wirtembergh; duca di Wirtimbergh</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -18628,7 +18628,7 @@
       <c r="D418" t="inlineStr"/>
       <c r="E418" t="inlineStr">
         <is>
-          <t>Don Luigi di Valasco; don Luigi di Velasco</t>
+          <t>Don Luigi di Valasco; don Luigi di Valasco; don Luigi di Velasco</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
@@ -18796,7 +18796,7 @@
       <c r="D422" t="inlineStr"/>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Henrico di Nassau; conte Henrico; principe Henrico di Nansau; principe Henrico fratello di sua Eccellenza; signor principe Henrico</t>
+          <t>Henrico di Nassau; conte Henrico; principe Henrico di Nansau; principe Henrico di Nassau; principe Henrico fratello di sua Eccellenza; signor principe Henrico</t>
         </is>
       </c>
       <c r="F422" t="inlineStr"/>
@@ -19614,7 +19614,7 @@
       <c r="D442" t="inlineStr"/>
       <c r="E442" t="inlineStr">
         <is>
-          <t>Hage; Hages; ambasciator Aghe; ambasciator Aghes; ambasciator Haghes; ambasciator a Constantinopoli; ambasciatore a Constantinopoli; nostro Hage; signor Haghes; signor Hayes</t>
+          <t>Hage; Hages; ambasciator Aghe; ambasciator Aghes; ambasciator Haghes; ambasciator a Constantinopoli; ambasciator in Constantinopoli; ambasciatore a Constantinopoli; nostro Hage; signor Haghes; signor Hayes</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
@@ -20128,7 +20128,7 @@
       <c r="D455" t="inlineStr"/>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Lantgravio di Hassia; landgravio Mauritio di Hessia; lantgrave Mauricio di Hassia; lantgravio di Assia; lantgravio di Hassia; marchese di Armenstat; marchese di Darmenstat</t>
+          <t>Lantgravio di Hassia; landgravio Mauritio di Hessia; langravio di Hassia; lantgrave Mauricio di Hassia; lantgravio di Assia; lantgravio di Hassia; marchese di Armenstat; marchese di Darmenstat</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
@@ -20564,7 +20564,7 @@
       <c r="D465" t="inlineStr"/>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Bucorst; Nicolo de Bucorst; Nicolo de Bucorst signor di Vimmenon; Nicolò de Bucorse signor di Vimenon; monsignor Bucorst; signor Bocorst; signor Bucorst</t>
+          <t>Bocorst; Buchorst; Bucorse; Bucorst; Nicolo de Bucorst; Nicolo de Bucorst signor di Vimmenon; Nicolò de Bucorse signor di Vimenon; monsignor Bucorst; signor Bocorst; signor Bucorst</t>
         </is>
       </c>
       <c r="F465" t="inlineStr">
@@ -20614,7 +20614,7 @@
       <c r="D466" t="inlineStr"/>
       <c r="E466" t="inlineStr">
         <is>
-          <t>pressidente di Frisia</t>
+          <t>presidente di Frisia; pressidente di Frisia; residente di Frisia</t>
         </is>
       </c>
       <c r="F466" t="inlineStr">
@@ -20762,7 +20762,7 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Van der Horst; Vander Hoot; Vander Horst; signor Vander Horst gentilhuomo principale di Gheldria</t>
+          <t>Van der Horst; Vander Horst; signor Vander Horst gentilhuomo principale di Gheldria</t>
         </is>
       </c>
       <c r="F470" t="inlineStr">
@@ -20964,7 +20964,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>monsignor di Brederod; signor di Brederod; signori di Brederod</t>
+          <t>signor di Brederod; signor di Bredevod; signori di Brederod</t>
         </is>
       </c>
       <c r="F475" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Ambasciator a Londra; ambasciator Lando; ambasciator sudetto d ’ Inghilterra</t>
+          <t>Ambasciator a Londra; Ambasciator in Londra; ambasciator Lando; ambasciator sudetto d ’ Inghilterra; ambasciatore Lando</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -26372,7 +26372,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>monsignor di Brederod; signor di Brederod; signori di Brederod</t>
+          <t>signor di Brederod; signor di Bredevod; signori di Brederod</t>
         </is>
       </c>
       <c r="F602" t="inlineStr">
@@ -28886,7 +28886,7 @@
       <c r="D661" t="inlineStr"/>
       <c r="E661" t="inlineStr">
         <is>
-          <t>Bernardino Rota; Bernardino Rotta; Rota; Rotta; al Rotta; capitan Bernardino Rota; capitan Bernardino Rotta; capitan Rota; capitano Bernardino Rota; capitano Rota; del Rotta; esso Rotta; il Rotta</t>
+          <t>Bernardino Rota; Bernardino Rotta; Rota; Rotta; al Rotta; capitan Bernardino Rota; capitan Bernardino Rotta; capitan Rota; capitano Bernardino Rota; capitano Rota; del Rota; del Rotta; esso Rota; esso Rotta; il Rotta</t>
         </is>
       </c>
       <c r="F661" t="inlineStr">
@@ -33875,7 +33875,7 @@
       <c r="D774" t="inlineStr"/>
       <c r="E774" t="inlineStr">
         <is>
-          <t>capitan Tomas Viller; capitan Tomas Ziller</t>
+          <t>capitan Tomas Viller</t>
         </is>
       </c>
       <c r="F774" t="inlineStr">
@@ -34115,7 +34115,7 @@
       <c r="D779" t="inlineStr"/>
       <c r="E779" t="inlineStr">
         <is>
-          <t>Baron di Chicester; Chichester; Chichiester; Chiester; ambasciator Chichiester; baron Chicester; baron Chichiester; milord Chicester</t>
+          <t>Baron di Chicester; Chichester; Chichiester; ambasciator Chichiester; baron Chicester; baron Chichiester; milord Chicester</t>
         </is>
       </c>
       <c r="F779" t="inlineStr">

</xml_diff>